<commit_message>
Sync planning SharePoint : S31
</commit_message>
<xml_diff>
--- a/Plannings 2026 S31.xlsx
+++ b/Plannings 2026 S31.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdalpes.sharepoint.com/sites/msteams_bd0f90/Documents partages/02. USP - TOS - General/RH/Plannings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5DA7E5F2-5163-46B7-B3E7-5E948235F29F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{5DA7E5F2-5163-46B7-B3E7-5E948235F29F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5CF791F7-8646-444A-BB39-BB2C9132AA58}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,20 @@
     <sheet name="Résultats par salarié" sheetId="2" r:id="rId2"/>
     <sheet name="Informations" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -446,7 +459,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -690,11 +703,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -831,6 +870,12 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1519,13 +1564,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1563,13 +1608,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1607,13 +1652,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1651,13 +1696,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1695,13 +1740,13 @@
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1739,13 +1784,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1783,13 +1828,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>31</xdr:row>
+      <xdr:row>32</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>31</xdr:row>
+      <xdr:row>32</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1827,13 +1872,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>31</xdr:row>
+      <xdr:row>32</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>31</xdr:row>
+      <xdr:row>32</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1871,13 +1916,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>31</xdr:row>
+      <xdr:row>32</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>31</xdr:row>
+      <xdr:row>32</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1915,13 +1960,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>33</xdr:row>
+      <xdr:row>34</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>33</xdr:row>
+      <xdr:row>34</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1959,13 +2004,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>33</xdr:row>
+      <xdr:row>34</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>33</xdr:row>
+      <xdr:row>34</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2003,13 +2048,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>33</xdr:row>
+      <xdr:row>34</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>33</xdr:row>
+      <xdr:row>34</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2047,13 +2092,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2091,13 +2136,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2135,13 +2180,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2179,13 +2224,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2223,13 +2268,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>42</xdr:row>
+      <xdr:row>43</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>42</xdr:row>
+      <xdr:row>43</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2267,13 +2312,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>42</xdr:row>
+      <xdr:row>43</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>42</xdr:row>
+      <xdr:row>43</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2311,13 +2356,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2355,13 +2400,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2399,13 +2444,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2443,13 +2488,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2487,13 +2532,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>40</xdr:row>
+      <xdr:row>41</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>40</xdr:row>
+      <xdr:row>41</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2531,13 +2576,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2573,147 +2618,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="42" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E7115008-A904-44DC-B183-635BC3D3A9E1}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1219200" y="8582025"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="43" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7B90405C-DCCB-424A-9E40-E2FAED652FFD}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3048000" y="8582025"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="44" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EAA6FBC6-C5B5-442F-8EF7-D0943FC21433}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3657600" y="8582025"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2751,13 +2664,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>29</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>29</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2958,6 +2871,270 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1219200" y="7629525"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="50" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BBC0105B-88FD-4EE3-AFB1-9E211F2D5CB5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3390900" y="5276850"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="51" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E5E714EE-0C58-44FB-B825-D3735717E92A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8477250" y="5276850"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="52" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{47EA545E-98A1-46B3-8EAB-DEAAA51B57CE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10172700" y="5276850"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="53" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F9FB6543-9CCE-480D-A5B8-7F24360A7356}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3390900" y="5276850"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="54" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E26F8661-E18C-4068-9D60-169E9CAF36B2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8477250" y="5276850"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="55" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{73E950CC-FC38-422C-8B77-5980283DE94B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10172700" y="5276850"/>
           <a:ext cx="123825" cy="123825"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3339,7 +3516,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="8" width="25.42578125" customWidth="1"/>
@@ -3688,96 +3865,94 @@
       <c r="G22" s="32"/>
       <c r="H22" s="33"/>
     </row>
-    <row r="23" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="14" t="s">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="46" t="s">
         <v>38</v>
       </c>
-      <c r="B23" s="31"/>
-      <c r="C23" s="32"/>
-      <c r="D23" s="32"/>
-      <c r="E23" s="32"/>
-      <c r="F23" s="32"/>
-      <c r="G23" s="32"/>
-      <c r="H23" s="33"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="38" t="s">
+      <c r="B23" s="15"/>
+      <c r="C23" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="D23" s="15"/>
+      <c r="E23" s="15"/>
+      <c r="F23" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G23" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="H23" s="16"/>
+    </row>
+    <row r="24" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="47"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H24" s="19"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="B24" s="15" t="s">
+      <c r="B25" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="C24" s="15"/>
-      <c r="D24" s="15" t="s">
+      <c r="C25" s="15"/>
+      <c r="D25" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="E24" s="15"/>
-      <c r="F24" s="15"/>
-      <c r="G24" s="15"/>
-      <c r="H24" s="16"/>
-    </row>
-    <row r="25" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="39"/>
-      <c r="B25" s="17" t="s">
+      <c r="E25" s="15"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="15"/>
+      <c r="H25" s="16"/>
+    </row>
+    <row r="26" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="39"/>
+      <c r="B26" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17" t="s">
+      <c r="C26" s="17"/>
+      <c r="D26" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
-      <c r="G25" s="17"/>
-      <c r="H25" s="18"/>
-    </row>
-    <row r="26" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="14" t="s">
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="17"/>
+      <c r="H26" s="18"/>
+    </row>
+    <row r="27" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="B26" s="31"/>
-      <c r="C26" s="32"/>
-      <c r="D26" s="32"/>
-      <c r="E26" s="32"/>
-      <c r="F26" s="32"/>
-      <c r="G26" s="32"/>
-      <c r="H26" s="33"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="38" t="s">
+      <c r="B27" s="31"/>
+      <c r="C27" s="32"/>
+      <c r="D27" s="32"/>
+      <c r="E27" s="32"/>
+      <c r="F27" s="32"/>
+      <c r="G27" s="32"/>
+      <c r="H27" s="33"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="B27" s="15"/>
-      <c r="C27" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="D27" s="15"/>
-      <c r="E27" s="15"/>
-      <c r="F27" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="G27" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="H27" s="29" t="s">
+      <c r="B28" s="15"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
+      <c r="H28" s="29" t="s">
         <v>88</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="40"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="H28" s="30" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
@@ -3788,117 +3963,117 @@
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
-      <c r="H29" s="28" t="s">
+      <c r="H29" s="30" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="40"/>
+      <c r="B30" s="2"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="28" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="39"/>
-      <c r="B30" s="17"/>
-      <c r="C30" s="17"/>
-      <c r="D30" s="17"/>
-      <c r="E30" s="17"/>
-      <c r="F30" s="17"/>
-      <c r="G30" s="17"/>
-      <c r="H30" s="18" t="s">
+    <row r="31" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="39"/>
+      <c r="B31" s="17"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17"/>
+      <c r="F31" s="17"/>
+      <c r="G31" s="17"/>
+      <c r="H31" s="18" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="14" t="s">
+    <row r="32" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B31" s="34"/>
-      <c r="C31" s="35"/>
-      <c r="D31" s="35"/>
-      <c r="E31" s="35"/>
-      <c r="F31" s="35"/>
-      <c r="G31" s="35"/>
-      <c r="H31" s="36"/>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="38" t="s">
+      <c r="B32" s="34"/>
+      <c r="C32" s="35"/>
+      <c r="D32" s="35"/>
+      <c r="E32" s="35"/>
+      <c r="F32" s="35"/>
+      <c r="G32" s="35"/>
+      <c r="H32" s="36"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="B32" s="15" t="s">
+      <c r="B33" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="C32" s="20" t="s">
+      <c r="C33" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="D32" s="15"/>
-      <c r="E32" s="15" t="s">
+      <c r="D33" s="15"/>
+      <c r="E33" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="F32" s="15"/>
-      <c r="G32" s="15"/>
-      <c r="H32" s="16"/>
-    </row>
-    <row r="33" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="41"/>
-      <c r="B33" s="2" t="s">
+      <c r="F33" s="15"/>
+      <c r="G33" s="15"/>
+      <c r="H33" s="16"/>
+    </row>
+    <row r="34" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="41"/>
+      <c r="B34" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C33" s="22" t="s">
+      <c r="C34" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2" t="s">
+      <c r="D34" s="2"/>
+      <c r="E34" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-      <c r="H33" s="19"/>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="38" t="s">
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
+      <c r="H34" s="19"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="38" t="s">
         <v>53</v>
       </c>
-      <c r="B34" s="15"/>
-      <c r="C34" s="15" t="s">
+      <c r="B35" s="15"/>
+      <c r="C35" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="D34" s="15"/>
-      <c r="E34" s="15" t="s">
+      <c r="D35" s="15"/>
+      <c r="E35" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="F34" s="15" t="s">
+      <c r="F35" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="G34" s="15"/>
-      <c r="H34" s="16"/>
-    </row>
-    <row r="35" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="39"/>
-      <c r="B35" s="17"/>
-      <c r="C35" s="17" t="s">
+      <c r="G35" s="15"/>
+      <c r="H35" s="16"/>
+    </row>
+    <row r="36" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="39"/>
+      <c r="B36" s="17"/>
+      <c r="C36" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="D35" s="17"/>
-      <c r="E35" s="17" t="s">
+      <c r="D36" s="17"/>
+      <c r="E36" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="F35" s="17" t="s">
+      <c r="F36" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="G35" s="17"/>
-      <c r="H35" s="18"/>
-    </row>
-    <row r="36" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="B36" s="34"/>
-      <c r="C36" s="35"/>
-      <c r="D36" s="35"/>
-      <c r="E36" s="35"/>
-      <c r="F36" s="35"/>
-      <c r="G36" s="35"/>
-      <c r="H36" s="36"/>
+      <c r="G36" s="17"/>
+      <c r="H36" s="18"/>
     </row>
     <row r="37" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="14" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B37" s="34"/>
       <c r="C37" s="35"/>
@@ -3910,7 +4085,7 @@
     </row>
     <row r="38" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="14" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B38" s="34"/>
       <c r="C38" s="35"/>
@@ -3920,117 +4095,117 @@
       <c r="G38" s="35"/>
       <c r="H38" s="36"/>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A39" s="38" t="s">
+    <row r="39" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="B39" s="34"/>
+      <c r="C39" s="35"/>
+      <c r="D39" s="35"/>
+      <c r="E39" s="35"/>
+      <c r="F39" s="35"/>
+      <c r="G39" s="35"/>
+      <c r="H39" s="36"/>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" s="38" t="s">
         <v>58</v>
       </c>
-      <c r="B39" s="3" t="s">
+      <c r="B40" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C39" s="2"/>
-      <c r="D39" s="3" t="s">
+      <c r="C40" s="2"/>
+      <c r="D40" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E39" s="3" t="s">
+      <c r="E40" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="F39" s="26" t="s">
+      <c r="F40" s="26" t="s">
         <v>86</v>
       </c>
-      <c r="G39" s="2"/>
-      <c r="H39" s="3" t="s">
+      <c r="G40" s="2"/>
+      <c r="H40" s="3" t="s">
         <v>17</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="40"/>
-      <c r="B40" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C40" s="2"/>
-      <c r="D40" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="F40" s="27" t="s">
-        <v>87</v>
-      </c>
-      <c r="G40" s="2"/>
-      <c r="H40" s="2" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="40"/>
-      <c r="B41" s="2"/>
+      <c r="B41" s="2" t="s">
+        <v>59</v>
+      </c>
       <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
-      <c r="E41" s="2"/>
-      <c r="F41" s="3" t="s">
-        <v>17</v>
+      <c r="D41" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F41" s="27" t="s">
+        <v>87</v>
       </c>
       <c r="G41" s="2"/>
-      <c r="H41" s="2"/>
-    </row>
-    <row r="42" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="39"/>
+      <c r="H41" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" s="40"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
-      <c r="F42" s="2" t="s">
-        <v>19</v>
+      <c r="F42" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="G42" s="2"/>
       <c r="H42" s="2"/>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43" s="38" t="s">
+    <row r="43" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="39"/>
+      <c r="B43" s="2"/>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2"/>
+      <c r="F43" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G43" s="2"/>
+      <c r="H43" s="2"/>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" s="38" t="s">
         <v>60</v>
       </c>
-      <c r="B43" s="15"/>
-      <c r="C43" s="20" t="s">
+      <c r="B44" s="15"/>
+      <c r="C44" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="D43" s="15"/>
-      <c r="E43" s="15"/>
-      <c r="F43" s="15"/>
-      <c r="G43" s="15"/>
-      <c r="H43" s="16" t="s">
+      <c r="D44" s="15"/>
+      <c r="E44" s="15"/>
+      <c r="F44" s="15"/>
+      <c r="G44" s="15"/>
+      <c r="H44" s="16" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="39"/>
-      <c r="B44" s="17"/>
-      <c r="C44" s="21" t="s">
+    <row r="45" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="39"/>
+      <c r="B45" s="17"/>
+      <c r="C45" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="D44" s="17"/>
-      <c r="E44" s="17"/>
-      <c r="F44" s="17"/>
-      <c r="G44" s="17"/>
-      <c r="H44" s="18" t="s">
+      <c r="D45" s="17"/>
+      <c r="E45" s="17"/>
+      <c r="F45" s="17"/>
+      <c r="G45" s="17"/>
+      <c r="H45" s="18" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="45" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="B45" s="34"/>
-      <c r="C45" s="35"/>
-      <c r="D45" s="35"/>
-      <c r="E45" s="35"/>
-      <c r="F45" s="35"/>
-      <c r="G45" s="35"/>
-      <c r="H45" s="36"/>
     </row>
     <row r="46" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="14" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B46" s="34"/>
       <c r="C46" s="35"/>
@@ -4042,7 +4217,7 @@
     </row>
     <row r="47" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B47" s="34"/>
       <c r="C47" s="35"/>
@@ -4052,39 +4227,51 @@
       <c r="G47" s="35"/>
       <c r="H47" s="36"/>
     </row>
-    <row r="48" spans="1:8" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="37"/>
-      <c r="C48" s="37"/>
-      <c r="D48" s="37"/>
-      <c r="E48" s="37"/>
-      <c r="F48" s="37"/>
-      <c r="G48" s="37"/>
-      <c r="H48" s="37"/>
+    <row r="48" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="B48" s="34"/>
+      <c r="C48" s="35"/>
+      <c r="D48" s="35"/>
+      <c r="E48" s="35"/>
+      <c r="F48" s="35"/>
+      <c r="G48" s="35"/>
+      <c r="H48" s="36"/>
+    </row>
+    <row r="49" spans="2:8" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B49" s="37"/>
+      <c r="C49" s="37"/>
+      <c r="D49" s="37"/>
+      <c r="E49" s="37"/>
+      <c r="F49" s="37"/>
+      <c r="G49" s="37"/>
+      <c r="H49" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="A25:A26"/>
     <mergeCell ref="A12:A13"/>
     <mergeCell ref="A15:A20"/>
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="B1:F1"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="A5:A8"/>
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="A39:A42"/>
-    <mergeCell ref="A27:A30"/>
-    <mergeCell ref="A32:A33"/>
-    <mergeCell ref="B48:H48"/>
-    <mergeCell ref="B36:H36"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A44:A45"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="A40:A43"/>
+    <mergeCell ref="A28:A31"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="B49:H49"/>
     <mergeCell ref="B37:H37"/>
     <mergeCell ref="B38:H38"/>
-    <mergeCell ref="B31:H31"/>
-    <mergeCell ref="B45:H45"/>
+    <mergeCell ref="B39:H39"/>
+    <mergeCell ref="B32:H32"/>
     <mergeCell ref="B46:H46"/>
     <mergeCell ref="B47:H47"/>
-    <mergeCell ref="B26:H26"/>
-    <mergeCell ref="B23:H23"/>
+    <mergeCell ref="B48:H48"/>
+    <mergeCell ref="B27:H27"/>
     <mergeCell ref="B22:H22"/>
     <mergeCell ref="B21:H21"/>
     <mergeCell ref="B9:H9"/>
@@ -4849,13 +5036,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{933B588B-C5B2-40BD-A3C5-CDAE89B816EC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CFAF909-22CD-4C2B-B7F8-3D90DB5F6BA5}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE388AC0-9D52-48E8-B910-EF1ED774E661}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D0B3754-6C75-46E2-AEB6-320755430F5B}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4EB77EF3-DE06-4A05-B168-33B2C1422B0E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91BE4166-D944-46DF-B4A1-0F13B5982209}"/>
 </file>
</xml_diff>